<commit_message>
Bornera en columna al frente (MOXA), Reprocesar rearma el instructivo, /api/version y correcciones del mapeo del PAE
Trabajo de otra sesion (2026-10-07, sin commitear hasta hoy), commiteado tal cual para juntarlo con el plan modular:
- instructivo / ruteo: bornera en columna al frente (catalogo 'columna_frente', mapeo lay['bornes_salida']): los
  cables salen en horizontal a la canaleta vertical del costado y se cablean seguidos de arriba a abajo
  (enganche_lateral, lado_paso).
- web: Reprocesar vuelve a armar el instructivo si hay topografico; /api/version (firma del codigo) y cierre del
  servidor viejo al abrir el programa con codigo nuevo.
- Mapeo verificado del PAE: 41XEX de 1 a 12 en orden y 11SK1 N-PE-L (correcciones_riel3_lateral.json, reexportado);
  bases base_76884 y base_tpt_ronda3 y probar_ronda3 al dia; CLAUDE.md.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/2 - Resultados/76884 mSafe2+ PAE/Mapeo de cables mSafe2+ PAE (ZPL-76884).xlsx
+++ b/2 - Resultados/76884 mSafe2+ PAE/Mapeo de cables mSafe2+ PAE (ZPL-76884).xlsx
@@ -716,7 +716,6 @@
           <t>alta</t>
         </is>
       </c>
-      <c r="N2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -782,7 +781,6 @@
           <t>alta</t>
         </is>
       </c>
-      <c r="N3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -848,7 +846,6 @@
           <t>alta</t>
         </is>
       </c>
-      <c r="N4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -914,7 +911,6 @@
           <t>alta</t>
         </is>
       </c>
-      <c r="N5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -980,7 +976,6 @@
           <t>alta</t>
         </is>
       </c>
-      <c r="N6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -1046,7 +1041,6 @@
           <t>alta</t>
         </is>
       </c>
-      <c r="N7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -1112,7 +1106,6 @@
           <t>alta</t>
         </is>
       </c>
-      <c r="N8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -1178,7 +1171,6 @@
           <t>alta</t>
         </is>
       </c>
-      <c r="N9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -1244,7 +1236,6 @@
           <t>alta</t>
         </is>
       </c>
-      <c r="N10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1310,7 +1301,6 @@
           <t>alta</t>
         </is>
       </c>
-      <c r="N11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1376,7 +1366,6 @@
           <t>alta</t>
         </is>
       </c>
-      <c r="N12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1432,13 +1421,11 @@
           <t>775.56, 627.41</t>
         </is>
       </c>
-      <c r="L13" t="inlineStr"/>
       <c r="M13" t="inlineStr">
         <is>
           <t>alta</t>
         </is>
       </c>
-      <c r="N13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -1504,7 +1491,6 @@
           <t>alta</t>
         </is>
       </c>
-      <c r="N14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1570,7 +1556,6 @@
           <t>alta</t>
         </is>
       </c>
-      <c r="N15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -1636,7 +1621,6 @@
           <t>alta</t>
         </is>
       </c>
-      <c r="N16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -1702,7 +1686,6 @@
           <t>alta</t>
         </is>
       </c>
-      <c r="N17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" s="3" t="inlineStr">
@@ -1828,13 +1811,11 @@
           <t>625.54, 487.81</t>
         </is>
       </c>
-      <c r="L19" t="inlineStr"/>
       <c r="M19" t="inlineStr">
         <is>
           <t>alta</t>
         </is>
       </c>
-      <c r="N19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -2030,13 +2011,11 @@
           <t>790.98, 635.40</t>
         </is>
       </c>
-      <c r="L22" t="inlineStr"/>
       <c r="M22" t="inlineStr">
         <is>
           <t>alta</t>
         </is>
       </c>
-      <c r="N22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -2092,13 +2071,11 @@
           <t>803.38, 635.40</t>
         </is>
       </c>
-      <c r="L23" t="inlineStr"/>
       <c r="M23" t="inlineStr">
         <is>
           <t>alta</t>
         </is>
       </c>
-      <c r="N23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -2154,13 +2131,11 @@
           <t>651.16, 541.93</t>
         </is>
       </c>
-      <c r="L24" t="inlineStr"/>
       <c r="M24" t="inlineStr">
         <is>
           <t>alta</t>
         </is>
       </c>
-      <c r="N24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -2216,13 +2191,11 @@
           <t>656.93, 541.93</t>
         </is>
       </c>
-      <c r="L25" t="inlineStr"/>
       <c r="M25" t="inlineStr">
         <is>
           <t>alta</t>
         </is>
       </c>
-      <c r="N25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -2288,7 +2261,6 @@
           <t>alta</t>
         </is>
       </c>
-      <c r="N26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -2354,7 +2326,6 @@
           <t>alta</t>
         </is>
       </c>
-      <c r="N27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" s="3" t="inlineStr">
@@ -2550,13 +2521,11 @@
           <t>651.16, 530.31</t>
         </is>
       </c>
-      <c r="L30" t="inlineStr"/>
       <c r="M30" t="inlineStr">
         <is>
           <t>alta</t>
         </is>
       </c>
-      <c r="N30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" s="3" t="inlineStr">
@@ -3252,7 +3221,6 @@
           <t>alta</t>
         </is>
       </c>
-      <c r="N40" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -3318,7 +3286,6 @@
           <t>alta</t>
         </is>
       </c>
-      <c r="N41" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -3384,7 +3351,6 @@
           <t>alta</t>
         </is>
       </c>
-      <c r="N42" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -3790,13 +3756,11 @@
           <t>823.79, 544.80</t>
         </is>
       </c>
-      <c r="L48" t="inlineStr"/>
       <c r="M48" t="inlineStr">
         <is>
           <t>alta</t>
         </is>
       </c>
-      <c r="N48" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -3852,13 +3816,11 @@
           <t>827.33, 544.80</t>
         </is>
       </c>
-      <c r="L49" t="inlineStr"/>
       <c r="M49" t="inlineStr">
         <is>
           <t>alta</t>
         </is>
       </c>
-      <c r="N49" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" s="3" t="inlineStr">
@@ -4046,13 +4008,11 @@
           <t>836.26, 544.80</t>
         </is>
       </c>
-      <c r="L52" t="inlineStr"/>
       <c r="M52" t="inlineStr">
         <is>
           <t>alta</t>
         </is>
       </c>
-      <c r="N52" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -4108,13 +4068,11 @@
           <t>839.80, 544.80</t>
         </is>
       </c>
-      <c r="L53" t="inlineStr"/>
       <c r="M53" t="inlineStr">
         <is>
           <t>alta</t>
         </is>
       </c>
-      <c r="N53" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -4170,13 +4128,11 @@
           <t>836.26, 551.17</t>
         </is>
       </c>
-      <c r="L54" t="inlineStr"/>
       <c r="M54" t="inlineStr">
         <is>
           <t>alta</t>
         </is>
       </c>
-      <c r="N54" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -4232,13 +4188,11 @@
           <t>839.80, 551.17</t>
         </is>
       </c>
-      <c r="L55" t="inlineStr"/>
       <c r="M55" t="inlineStr">
         <is>
           <t>alta</t>
         </is>
       </c>
-      <c r="N55" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -4294,13 +4248,11 @@
           <t>845.12, 544.80</t>
         </is>
       </c>
-      <c r="L56" t="inlineStr"/>
       <c r="M56" t="inlineStr">
         <is>
           <t>alta</t>
         </is>
       </c>
-      <c r="N56" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -4356,13 +4308,11 @@
           <t>848.66, 544.80</t>
         </is>
       </c>
-      <c r="L57" t="inlineStr"/>
       <c r="M57" t="inlineStr">
         <is>
           <t>alta</t>
         </is>
       </c>
-      <c r="N57" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -4418,13 +4368,11 @@
           <t>845.12, 551.17</t>
         </is>
       </c>
-      <c r="L58" t="inlineStr"/>
       <c r="M58" t="inlineStr">
         <is>
           <t>alta</t>
         </is>
       </c>
-      <c r="N58" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
@@ -4480,13 +4428,11 @@
           <t>848.66, 551.17</t>
         </is>
       </c>
-      <c r="L59" t="inlineStr"/>
       <c r="M59" t="inlineStr">
         <is>
           <t>alta</t>
         </is>
       </c>
-      <c r="N59" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" s="3" t="inlineStr">
@@ -4806,13 +4752,11 @@
           <t>725.64, 413.66</t>
         </is>
       </c>
-      <c r="L64" t="inlineStr"/>
       <c r="M64" t="inlineStr">
         <is>
           <t>alta</t>
         </is>
       </c>
-      <c r="N64" t="inlineStr"/>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -4868,13 +4812,11 @@
           <t>732.94, 413.66</t>
         </is>
       </c>
-      <c r="L65" t="inlineStr"/>
       <c r="M65" t="inlineStr">
         <is>
           <t>alta</t>
         </is>
       </c>
-      <c r="N65" t="inlineStr"/>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
@@ -4930,13 +4872,11 @@
           <t>725.64, 402.41</t>
         </is>
       </c>
-      <c r="L66" t="inlineStr"/>
       <c r="M66" t="inlineStr">
         <is>
           <t>alta</t>
         </is>
       </c>
-      <c r="N66" t="inlineStr"/>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
@@ -4992,13 +4932,11 @@
           <t>732.94, 402.41</t>
         </is>
       </c>
-      <c r="L67" t="inlineStr"/>
       <c r="M67" t="inlineStr">
         <is>
           <t>alta</t>
         </is>
       </c>
-      <c r="N67" t="inlineStr"/>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
@@ -5194,13 +5132,11 @@
           <t>823.79, 551.17</t>
         </is>
       </c>
-      <c r="L70" t="inlineStr"/>
       <c r="M70" t="inlineStr">
         <is>
           <t>alta</t>
         </is>
       </c>
-      <c r="N70" t="inlineStr"/>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
@@ -5256,13 +5192,11 @@
           <t>827.33, 551.17</t>
         </is>
       </c>
-      <c r="L71" t="inlineStr"/>
       <c r="M71" t="inlineStr">
         <is>
           <t>alta</t>
         </is>
       </c>
-      <c r="N71" t="inlineStr"/>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
@@ -5318,7 +5252,6 @@
           <t>888.77, 691.72</t>
         </is>
       </c>
-      <c r="L72" t="inlineStr"/>
       <c r="M72" t="inlineStr">
         <is>
           <t>alta</t>
@@ -5922,7 +5855,6 @@
           <t>alta</t>
         </is>
       </c>
-      <c r="N81" t="inlineStr"/>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
@@ -5988,7 +5920,6 @@
           <t>alta</t>
         </is>
       </c>
-      <c r="N82" t="inlineStr"/>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
@@ -6054,7 +5985,6 @@
           <t>alta</t>
         </is>
       </c>
-      <c r="N83" t="inlineStr"/>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
@@ -6120,7 +6050,6 @@
           <t>alta</t>
         </is>
       </c>
-      <c r="N84" t="inlineStr"/>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
@@ -6186,7 +6115,6 @@
           <t>alta</t>
         </is>
       </c>
-      <c r="N85" t="inlineStr"/>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
@@ -6252,7 +6180,6 @@
           <t>alta</t>
         </is>
       </c>
-      <c r="N86" t="inlineStr"/>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
@@ -6318,7 +6245,6 @@
           <t>alta</t>
         </is>
       </c>
-      <c r="N87" t="inlineStr"/>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
@@ -6384,7 +6310,6 @@
           <t>alta</t>
         </is>
       </c>
-      <c r="N88" t="inlineStr"/>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
@@ -6450,7 +6375,6 @@
           <t>alta</t>
         </is>
       </c>
-      <c r="N89" t="inlineStr"/>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
@@ -6516,7 +6440,6 @@
           <t>alta</t>
         </is>
       </c>
-      <c r="N90" t="inlineStr"/>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
@@ -6582,7 +6505,6 @@
           <t>alta</t>
         </is>
       </c>
-      <c r="N91" t="inlineStr"/>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
@@ -6648,7 +6570,6 @@
           <t>alta</t>
         </is>
       </c>
-      <c r="N92" t="inlineStr"/>
     </row>
     <row r="93">
       <c r="A93" s="3" t="inlineStr">
@@ -6984,13 +6905,11 @@
           <t>842.03, 687.10</t>
         </is>
       </c>
-      <c r="L97" t="inlineStr"/>
       <c r="M97" t="inlineStr">
         <is>
           <t>alta</t>
         </is>
       </c>
-      <c r="N97" t="inlineStr"/>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
@@ -7046,13 +6965,11 @@
           <t>853.63, 679.91</t>
         </is>
       </c>
-      <c r="L98" t="inlineStr"/>
       <c r="M98" t="inlineStr">
         <is>
           <t>alta</t>
         </is>
       </c>
-      <c r="N98" t="inlineStr"/>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
@@ -7118,7 +7035,6 @@
           <t>alta</t>
         </is>
       </c>
-      <c r="N99" t="inlineStr"/>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
@@ -7184,7 +7100,6 @@
           <t>alta</t>
         </is>
       </c>
-      <c r="N100" t="inlineStr"/>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
@@ -7250,7 +7165,6 @@
           <t>alta</t>
         </is>
       </c>
-      <c r="N101" t="inlineStr"/>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
@@ -7316,7 +7230,6 @@
           <t>alta</t>
         </is>
       </c>
-      <c r="N102" t="inlineStr"/>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
@@ -7382,7 +7295,6 @@
           <t>alta</t>
         </is>
       </c>
-      <c r="N103" t="inlineStr"/>
     </row>
     <row r="104">
       <c r="A104" s="3" t="inlineStr">
@@ -7928,13 +7840,11 @@
           <t>709.73, 487.81</t>
         </is>
       </c>
-      <c r="L111" t="inlineStr"/>
       <c r="M111" t="inlineStr">
         <is>
           <t>alta</t>
         </is>
       </c>
-      <c r="N111" t="inlineStr"/>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
@@ -7990,13 +7900,11 @@
           <t>715.50, 487.81</t>
         </is>
       </c>
-      <c r="L112" t="inlineStr"/>
       <c r="M112" t="inlineStr">
         <is>
           <t>alta</t>
         </is>
       </c>
-      <c r="N112" t="inlineStr"/>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
@@ -8052,13 +7960,11 @@
           <t>721.28, 487.81</t>
         </is>
       </c>
-      <c r="L113" t="inlineStr"/>
       <c r="M113" t="inlineStr">
         <is>
           <t>alta</t>
         </is>
       </c>
-      <c r="N113" t="inlineStr"/>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
@@ -8114,13 +8020,11 @@
           <t>735.35, 487.81</t>
         </is>
       </c>
-      <c r="L114" t="inlineStr"/>
       <c r="M114" t="inlineStr">
         <is>
           <t>alta</t>
         </is>
       </c>
-      <c r="N114" t="inlineStr"/>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
@@ -8176,13 +8080,11 @@
           <t>741.12, 499.43</t>
         </is>
       </c>
-      <c r="L115" t="inlineStr"/>
       <c r="M115" t="inlineStr">
         <is>
           <t>alta</t>
         </is>
       </c>
-      <c r="N115" t="inlineStr"/>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
@@ -8238,13 +8140,11 @@
           <t>741.12, 487.81</t>
         </is>
       </c>
-      <c r="L116" t="inlineStr"/>
       <c r="M116" t="inlineStr">
         <is>
           <t>alta</t>
         </is>
       </c>
-      <c r="N116" t="inlineStr"/>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
@@ -8532,8 +8432,6 @@
           <t>(sin número)</t>
         </is>
       </c>
-      <c r="B121" t="inlineStr"/>
-      <c r="C121" t="inlineStr"/>
       <c r="D121" t="inlineStr">
         <is>
           <t>E6</t>
@@ -8574,13 +8472,11 @@
           <t>689.95, 355.55</t>
         </is>
       </c>
-      <c r="L121" t="inlineStr"/>
       <c r="M121" t="inlineStr">
         <is>
           <t>alta</t>
         </is>
       </c>
-      <c r="N121" t="inlineStr"/>
     </row>
     <row r="122">
       <c r="A122" t="inlineStr">
@@ -8588,8 +8484,6 @@
           <t>(sin número)</t>
         </is>
       </c>
-      <c r="B122" t="inlineStr"/>
-      <c r="C122" t="inlineStr"/>
       <c r="D122" t="inlineStr">
         <is>
           <t>E6</t>
@@ -8630,13 +8524,11 @@
           <t>689.95, 366.94</t>
         </is>
       </c>
-      <c r="L122" t="inlineStr"/>
       <c r="M122" t="inlineStr">
         <is>
           <t>alta</t>
         </is>
       </c>
-      <c r="N122" t="inlineStr"/>
     </row>
     <row r="123">
       <c r="A123" t="inlineStr">
@@ -8644,8 +8536,6 @@
           <t>(sin número)</t>
         </is>
       </c>
-      <c r="B123" t="inlineStr"/>
-      <c r="C123" t="inlineStr"/>
       <c r="D123" t="inlineStr">
         <is>
           <t>E6</t>
@@ -8686,13 +8576,11 @@
           <t>694.17, 364.26</t>
         </is>
       </c>
-      <c r="L123" t="inlineStr"/>
       <c r="M123" t="inlineStr">
         <is>
           <t>alta</t>
         </is>
       </c>
-      <c r="N123" t="inlineStr"/>
     </row>
     <row r="124">
       <c r="A124" t="inlineStr">
@@ -8700,8 +8588,6 @@
           <t>(sin número)</t>
         </is>
       </c>
-      <c r="B124" t="inlineStr"/>
-      <c r="C124" t="inlineStr"/>
       <c r="D124" t="inlineStr">
         <is>
           <t>E6</t>
@@ -8742,13 +8628,11 @@
           <t>823.04, 355.43</t>
         </is>
       </c>
-      <c r="L124" t="inlineStr"/>
       <c r="M124" t="inlineStr">
         <is>
           <t>alta</t>
         </is>
       </c>
-      <c r="N124" t="inlineStr"/>
     </row>
     <row r="125">
       <c r="A125" t="inlineStr">
@@ -8756,8 +8640,6 @@
           <t>(sin número)</t>
         </is>
       </c>
-      <c r="B125" t="inlineStr"/>
-      <c r="C125" t="inlineStr"/>
       <c r="D125" t="inlineStr">
         <is>
           <t>E6</t>
@@ -8798,13 +8680,11 @@
           <t>823.04, 366.82</t>
         </is>
       </c>
-      <c r="L125" t="inlineStr"/>
       <c r="M125" t="inlineStr">
         <is>
           <t>alta</t>
         </is>
       </c>
-      <c r="N125" t="inlineStr"/>
     </row>
     <row r="126">
       <c r="A126" t="inlineStr">
@@ -8817,7 +8697,6 @@
           <t>Verde/amarillo</t>
         </is>
       </c>
-      <c r="C126" t="inlineStr"/>
       <c r="D126" t="inlineStr">
         <is>
           <t>E6</t>
@@ -8843,13 +8722,11 @@
           <t>Bandeja principal</t>
         </is>
       </c>
-      <c r="J126" t="inlineStr"/>
       <c r="K126" t="inlineStr">
         <is>
           <t>830.91, 364.14</t>
         </is>
       </c>
-      <c r="L126" t="inlineStr"/>
       <c r="M126" t="inlineStr">
         <is>
           <t>alta</t>
@@ -8867,8 +8744,6 @@
           <t>(sin número)</t>
         </is>
       </c>
-      <c r="B127" t="inlineStr"/>
-      <c r="C127" t="inlineStr"/>
       <c r="D127" t="inlineStr">
         <is>
           <t>E6</t>
@@ -8909,13 +8784,11 @@
           <t>842.85, 355.43</t>
         </is>
       </c>
-      <c r="L127" t="inlineStr"/>
       <c r="M127" t="inlineStr">
         <is>
           <t>alta</t>
         </is>
       </c>
-      <c r="N127" t="inlineStr"/>
     </row>
     <row r="128">
       <c r="A128" t="inlineStr">
@@ -8923,8 +8796,6 @@
           <t>(sin número)</t>
         </is>
       </c>
-      <c r="B128" t="inlineStr"/>
-      <c r="C128" t="inlineStr"/>
       <c r="D128" t="inlineStr">
         <is>
           <t>E6</t>
@@ -8965,13 +8836,11 @@
           <t>853.80, 366.82</t>
         </is>
       </c>
-      <c r="L128" t="inlineStr"/>
       <c r="M128" t="inlineStr">
         <is>
           <t>alta</t>
         </is>
       </c>
-      <c r="N128" t="inlineStr"/>
     </row>
     <row r="129">
       <c r="A129" t="inlineStr">
@@ -8979,8 +8848,6 @@
           <t>(sin número)</t>
         </is>
       </c>
-      <c r="B129" t="inlineStr"/>
-      <c r="C129" t="inlineStr"/>
       <c r="D129" t="inlineStr">
         <is>
           <t>E6</t>
@@ -9021,13 +8888,11 @@
           <t>861.10, 355.43</t>
         </is>
       </c>
-      <c r="L129" t="inlineStr"/>
       <c r="M129" t="inlineStr">
         <is>
           <t>alta</t>
         </is>
       </c>
-      <c r="N129" t="inlineStr"/>
     </row>
     <row r="130">
       <c r="A130" t="inlineStr">
@@ -9035,8 +8900,6 @@
           <t>(sin número)</t>
         </is>
       </c>
-      <c r="B130" t="inlineStr"/>
-      <c r="C130" t="inlineStr"/>
       <c r="D130" t="inlineStr">
         <is>
           <t>E6</t>
@@ -9077,13 +8940,11 @@
           <t>861.10, 366.82</t>
         </is>
       </c>
-      <c r="L130" t="inlineStr"/>
       <c r="M130" t="inlineStr">
         <is>
           <t>alta</t>
         </is>
       </c>
-      <c r="N130" t="inlineStr"/>
     </row>
     <row r="131">
       <c r="A131" t="inlineStr">
@@ -9091,8 +8952,6 @@
           <t>(sin número)</t>
         </is>
       </c>
-      <c r="B131" t="inlineStr"/>
-      <c r="C131" t="inlineStr"/>
       <c r="D131" t="inlineStr">
         <is>
           <t>E6</t>
@@ -9133,13 +8992,11 @@
           <t>842.85, 366.82</t>
         </is>
       </c>
-      <c r="L131" t="inlineStr"/>
       <c r="M131" t="inlineStr">
         <is>
           <t>alta</t>
         </is>
       </c>
-      <c r="N131" t="inlineStr"/>
     </row>
     <row r="132">
       <c r="A132" t="inlineStr">
@@ -9147,8 +9004,6 @@
           <t>(sin número)</t>
         </is>
       </c>
-      <c r="B132" t="inlineStr"/>
-      <c r="C132" t="inlineStr"/>
       <c r="D132" t="inlineStr">
         <is>
           <t>E6</t>
@@ -9189,13 +9044,11 @@
           <t>846.50, 355.43</t>
         </is>
       </c>
-      <c r="L132" t="inlineStr"/>
       <c r="M132" t="inlineStr">
         <is>
           <t>alta</t>
         </is>
       </c>
-      <c r="N132" t="inlineStr"/>
     </row>
     <row r="133">
       <c r="A133" t="inlineStr">
@@ -9203,8 +9056,6 @@
           <t>(sin número)</t>
         </is>
       </c>
-      <c r="B133" t="inlineStr"/>
-      <c r="C133" t="inlineStr"/>
       <c r="D133" t="inlineStr">
         <is>
           <t>E6</t>
@@ -9245,13 +9096,11 @@
           <t>846.50, 366.82</t>
         </is>
       </c>
-      <c r="L133" t="inlineStr"/>
       <c r="M133" t="inlineStr">
         <is>
           <t>alta</t>
         </is>
       </c>
-      <c r="N133" t="inlineStr"/>
     </row>
     <row r="134">
       <c r="A134" t="inlineStr">
@@ -9259,8 +9108,6 @@
           <t>(sin número)</t>
         </is>
       </c>
-      <c r="B134" t="inlineStr"/>
-      <c r="C134" t="inlineStr"/>
       <c r="D134" t="inlineStr">
         <is>
           <t>E6</t>
@@ -9301,13 +9148,11 @@
           <t>850.15, 355.43</t>
         </is>
       </c>
-      <c r="L134" t="inlineStr"/>
       <c r="M134" t="inlineStr">
         <is>
           <t>alta</t>
         </is>
       </c>
-      <c r="N134" t="inlineStr"/>
     </row>
     <row r="135">
       <c r="A135" t="inlineStr">
@@ -9315,8 +9160,6 @@
           <t>(sin número)</t>
         </is>
       </c>
-      <c r="B135" t="inlineStr"/>
-      <c r="C135" t="inlineStr"/>
       <c r="D135" t="inlineStr">
         <is>
           <t>E6</t>
@@ -9357,13 +9200,11 @@
           <t>850.15, 366.82</t>
         </is>
       </c>
-      <c r="L135" t="inlineStr"/>
       <c r="M135" t="inlineStr">
         <is>
           <t>alta</t>
         </is>
       </c>
-      <c r="N135" t="inlineStr"/>
     </row>
     <row r="136">
       <c r="A136" t="inlineStr">
@@ -9371,8 +9212,6 @@
           <t>(sin número)</t>
         </is>
       </c>
-      <c r="B136" t="inlineStr"/>
-      <c r="C136" t="inlineStr"/>
       <c r="D136" t="inlineStr">
         <is>
           <t>E6</t>
@@ -9413,13 +9252,11 @@
           <t>857.45, 355.43</t>
         </is>
       </c>
-      <c r="L136" t="inlineStr"/>
       <c r="M136" t="inlineStr">
         <is>
           <t>alta</t>
         </is>
       </c>
-      <c r="N136" t="inlineStr"/>
     </row>
     <row r="137">
       <c r="A137" t="inlineStr">
@@ -9427,8 +9264,6 @@
           <t>(sin número)</t>
         </is>
       </c>
-      <c r="B137" t="inlineStr"/>
-      <c r="C137" t="inlineStr"/>
       <c r="D137" t="inlineStr">
         <is>
           <t>E6</t>
@@ -9469,13 +9304,11 @@
           <t>857.45, 366.82</t>
         </is>
       </c>
-      <c r="L137" t="inlineStr"/>
       <c r="M137" t="inlineStr">
         <is>
           <t>alta</t>
         </is>
       </c>
-      <c r="N137" t="inlineStr"/>
     </row>
     <row r="138">
       <c r="A138" t="inlineStr">
@@ -9483,8 +9316,6 @@
           <t>(sin número)</t>
         </is>
       </c>
-      <c r="B138" t="inlineStr"/>
-      <c r="C138" t="inlineStr"/>
       <c r="D138" t="inlineStr">
         <is>
           <t>E6</t>
@@ -9525,13 +9356,11 @@
           <t>853.80, 355.43</t>
         </is>
       </c>
-      <c r="L138" t="inlineStr"/>
       <c r="M138" t="inlineStr">
         <is>
           <t>alta</t>
         </is>
       </c>
-      <c r="N138" t="inlineStr"/>
     </row>
     <row r="139">
       <c r="A139" t="inlineStr">
@@ -9544,7 +9373,6 @@
           <t>Apantallamiento</t>
         </is>
       </c>
-      <c r="C139" t="inlineStr"/>
       <c r="D139" t="inlineStr">
         <is>
           <t>E6</t>
@@ -9585,7 +9413,6 @@
           <t>729.29, 413.66</t>
         </is>
       </c>
-      <c r="L139" t="inlineStr"/>
       <c r="M139" t="inlineStr">
         <is>
           <t>alta</t>
@@ -9608,7 +9435,6 @@
           <t>Apantallamiento</t>
         </is>
       </c>
-      <c r="C140" t="inlineStr"/>
       <c r="D140" t="inlineStr">
         <is>
           <t>E6</t>
@@ -9649,7 +9475,6 @@
           <t>729.29, 402.41</t>
         </is>
       </c>
-      <c r="L140" t="inlineStr"/>
       <c r="M140" t="inlineStr">
         <is>
           <t>alta</t>
@@ -9672,7 +9497,6 @@
           <t>Verde/amarillo</t>
         </is>
       </c>
-      <c r="C141" t="inlineStr"/>
       <c r="D141" t="inlineStr">
         <is>
           <t>E6</t>
@@ -9698,13 +9522,11 @@
           <t>Bandeja principal</t>
         </is>
       </c>
-      <c r="J141" t="inlineStr"/>
       <c r="K141" t="inlineStr">
         <is>
           <t>740.23, 413.66</t>
         </is>
       </c>
-      <c r="L141" t="inlineStr"/>
       <c r="M141" t="inlineStr">
         <is>
           <t>alta</t>
@@ -9780,7 +9602,6 @@
           <t>alta</t>
         </is>
       </c>
-      <c r="N142" t="inlineStr"/>
     </row>
     <row r="143">
       <c r="A143" t="inlineStr">
@@ -9846,7 +9667,6 @@
           <t>alta</t>
         </is>
       </c>
-      <c r="N143" t="inlineStr"/>
     </row>
     <row r="144">
       <c r="A144" t="inlineStr">
@@ -9912,7 +9732,6 @@
           <t>alta</t>
         </is>
       </c>
-      <c r="N144" t="inlineStr"/>
     </row>
     <row r="145">
       <c r="A145" t="inlineStr">
@@ -9968,7 +9787,6 @@
           <t>354.32, 398.60</t>
         </is>
       </c>
-      <c r="L145" t="inlineStr"/>
       <c r="M145" t="inlineStr">
         <is>
           <t>alta</t>
@@ -10034,7 +9852,6 @@
           <t>360.10, 398.60</t>
         </is>
       </c>
-      <c r="L146" t="inlineStr"/>
       <c r="M146" t="inlineStr">
         <is>
           <t>alta</t>
@@ -10095,7 +9912,6 @@
           <t>Bandeja lateral izq.</t>
         </is>
       </c>
-      <c r="K147" t="inlineStr"/>
       <c r="L147" t="inlineStr">
         <is>
           <t>249.88, 408.15</t>
@@ -10161,7 +9977,6 @@
           <t>Bandeja lateral izq.</t>
         </is>
       </c>
-      <c r="K148" t="inlineStr"/>
       <c r="L148" t="inlineStr">
         <is>
           <t>237.26, 408.15</t>
@@ -10242,7 +10057,6 @@
           <t>alta</t>
         </is>
       </c>
-      <c r="N149" t="inlineStr"/>
     </row>
     <row r="150">
       <c r="A150" t="inlineStr">
@@ -10308,7 +10122,6 @@
           <t>alta</t>
         </is>
       </c>
-      <c r="N150" t="inlineStr"/>
     </row>
     <row r="151">
       <c r="A151" t="inlineStr">
@@ -10374,7 +10187,6 @@
           <t>alta</t>
         </is>
       </c>
-      <c r="N151" t="inlineStr"/>
     </row>
     <row r="152">
       <c r="A152" t="inlineStr">
@@ -10440,7 +10252,6 @@
           <t>alta</t>
         </is>
       </c>
-      <c r="N152" t="inlineStr"/>
     </row>
     <row r="153">
       <c r="A153" s="3" t="inlineStr">
@@ -10493,7 +10304,7 @@
       </c>
       <c r="K153" s="3" t="inlineStr">
         <is>
-          <t>208.29, 362.50</t>
+          <t>221.75, 362.50</t>
         </is>
       </c>
       <c r="L153" s="3" t="inlineStr">
@@ -10503,12 +10314,12 @@
       </c>
       <c r="M153" s="3" t="inlineStr">
         <is>
-          <t>media</t>
+          <t>alta</t>
         </is>
       </c>
       <c r="N153" s="3" t="inlineStr">
         <is>
-          <t>11SK1 L ABAJO: Phoenix EO-I/UT (toma tipo I, 45 x 75 mm, bornes a tornillo M3). Los 3 tornillos ranurados estan en la franja de ABAJO del dibujo (aros r 1.62 a y 362.5); regla del taller: 11SK1 todo por abajo. Orden supuesto L / PE / N</t>
+          <t>11SK1 L ABAJO: Phoenix EO-I/UT (toma tipo I, 45 x 75 mm, bornes a tornillo M3). Los 3 tornillos ranurados estan en la franja de ABAJO del dibujo (aros r 1.62 a y 362.5); regla del taller: 11SK1 todo por abajo. Orden supuesto L / PE / N Corregido por el taller el 2026-10-07: orden N / PE / L de izquierda a derecha (foto oficial Phoenix).</t>
         </is>
       </c>
     </row>
@@ -10563,7 +10374,7 @@
       </c>
       <c r="K154" s="3" t="inlineStr">
         <is>
-          <t>221.75, 362.50</t>
+          <t>208.29, 362.50</t>
         </is>
       </c>
       <c r="L154" s="3" t="inlineStr">
@@ -10573,12 +10384,12 @@
       </c>
       <c r="M154" s="3" t="inlineStr">
         <is>
-          <t>media</t>
+          <t>alta</t>
         </is>
       </c>
       <c r="N154" s="3" t="inlineStr">
         <is>
-          <t>11SK1 N ABAJO: Phoenix EO-I/UT (toma tipo I, 45 x 75 mm, bornes a tornillo M3). Los 3 tornillos ranurados estan en la franja de ABAJO del dibujo (aros r 1.62 a y 362.5); regla del taller: 11SK1 todo por abajo. Orden supuesto L / PE / N</t>
+          <t>11SK1 N ABAJO: Phoenix EO-I/UT (toma tipo I, 45 x 75 mm, bornes a tornillo M3). Los 3 tornillos ranurados estan en la franja de ABAJO del dibujo (aros r 1.62 a y 362.5); regla del taller: 11SK1 todo por abajo. Orden supuesto L / PE / N Corregido por el taller el 2026-10-07: orden N / PE / L de izquierda a derecha (foto oficial Phoenix).</t>
         </is>
       </c>
     </row>
@@ -10631,7 +10442,6 @@
           <t>Bandeja lateral izq.</t>
         </is>
       </c>
-      <c r="K155" t="inlineStr"/>
       <c r="L155" t="inlineStr">
         <is>
           <t>259.52, 516.65</t>
@@ -10642,7 +10452,6 @@
           <t>alta</t>
         </is>
       </c>
-      <c r="N155" t="inlineStr"/>
     </row>
     <row r="156">
       <c r="A156" s="3" t="inlineStr">
@@ -11113,10 +10922,6 @@
           <t>Fuera (puerta / campo)</t>
         </is>
       </c>
-      <c r="K162" t="inlineStr"/>
-      <c r="L162" t="inlineStr"/>
-      <c r="M162" t="inlineStr"/>
-      <c r="N162" t="inlineStr"/>
     </row>
     <row r="163">
       <c r="A163" t="inlineStr">
@@ -11167,10 +10972,6 @@
           <t>Fuera (puerta / campo)</t>
         </is>
       </c>
-      <c r="K163" t="inlineStr"/>
-      <c r="L163" t="inlineStr"/>
-      <c r="M163" t="inlineStr"/>
-      <c r="N163" t="inlineStr"/>
     </row>
     <row r="164">
       <c r="A164" t="inlineStr">
@@ -11221,10 +11022,6 @@
           <t>Fuera (puerta / campo)</t>
         </is>
       </c>
-      <c r="K164" t="inlineStr"/>
-      <c r="L164" t="inlineStr"/>
-      <c r="M164" t="inlineStr"/>
-      <c r="N164" t="inlineStr"/>
     </row>
     <row r="165">
       <c r="A165" t="inlineStr">
@@ -11275,10 +11072,6 @@
           <t>Fuera (puerta / campo)</t>
         </is>
       </c>
-      <c r="K165" t="inlineStr"/>
-      <c r="L165" t="inlineStr"/>
-      <c r="M165" t="inlineStr"/>
-      <c r="N165" t="inlineStr"/>
     </row>
     <row r="166">
       <c r="A166" t="inlineStr">
@@ -11329,7 +11122,6 @@
           <t>Bandeja lateral izq.</t>
         </is>
       </c>
-      <c r="K166" t="inlineStr"/>
       <c r="L166" t="inlineStr">
         <is>
           <t>282.63, 516.65</t>
@@ -11395,7 +11187,6 @@
           <t>Bandeja lateral izq.</t>
         </is>
       </c>
-      <c r="K167" t="inlineStr"/>
       <c r="L167" t="inlineStr">
         <is>
           <t>288.40, 516.65</t>
@@ -11418,8 +11209,6 @@
           <t>(sin número)</t>
         </is>
       </c>
-      <c r="B168" t="inlineStr"/>
-      <c r="C168" t="inlineStr"/>
       <c r="D168" t="inlineStr">
         <is>
           <t>LI ↔ LI (al montar)</t>
@@ -11455,10 +11244,6 @@
           <t>campo</t>
         </is>
       </c>
-      <c r="K168" t="inlineStr"/>
-      <c r="L168" t="inlineStr"/>
-      <c r="M168" t="inlineStr"/>
-      <c r="N168" t="inlineStr"/>
     </row>
     <row r="169">
       <c r="A169" t="inlineStr">
@@ -11466,8 +11251,6 @@
           <t>(sin número)</t>
         </is>
       </c>
-      <c r="B169" t="inlineStr"/>
-      <c r="C169" t="inlineStr"/>
       <c r="D169" t="inlineStr">
         <is>
           <t>LI ↔ LI (al montar)</t>
@@ -11503,10 +11286,6 @@
           <t>campo</t>
         </is>
       </c>
-      <c r="K169" t="inlineStr"/>
-      <c r="L169" t="inlineStr"/>
-      <c r="M169" t="inlineStr"/>
-      <c r="N169" t="inlineStr"/>
     </row>
     <row r="170">
       <c r="A170" s="3" t="inlineStr">
@@ -11569,12 +11348,12 @@
       </c>
       <c r="M170" s="3" t="inlineStr">
         <is>
-          <t>media</t>
+          <t>alta</t>
         </is>
       </c>
       <c r="N170" s="3" t="inlineStr">
         <is>
-          <t>11SK1 PE ABAJO: Phoenix EO-I/UT (toma tipo I, 45 x 75 mm, bornes a tornillo M3). Los 3 tornillos ranurados estan en la franja de ABAJO del dibujo (aros r 1.62 a y 362.5); regla del taller: 11SK1 todo por abajo. Orden supuesto L / PE / N</t>
+          <t>11SK1 PE ABAJO: Phoenix EO-I/UT (toma tipo I, 45 x 75 mm, bornes a tornillo M3). Los 3 tornillos ranurados estan en la franja de ABAJO del dibujo (aros r 1.62 a y 362.5); regla del taller: 11SK1 todo por abajo. Orden supuesto L / PE / N Corregido por el taller el 2026-10-07: orden N / PE / L de izquierda a derecha (foto oficial Phoenix).</t>
         </is>
       </c>
     </row>
@@ -11869,7 +11648,6 @@
           <t>Apantallamiento</t>
         </is>
       </c>
-      <c r="C175" t="inlineStr"/>
       <c r="D175" t="inlineStr">
         <is>
           <t>LI ↔ LI (al montar)</t>
@@ -11880,7 +11658,6 @@
           <t>21PCB01 37</t>
         </is>
       </c>
-      <c r="F175" t="inlineStr"/>
       <c r="G175" t="inlineStr">
         <is>
           <t>-21PCB01:37</t>
@@ -11891,10 +11668,6 @@
           <t>Fuera (puerta / campo)</t>
         </is>
       </c>
-      <c r="J175" t="inlineStr"/>
-      <c r="K175" t="inlineStr"/>
-      <c r="L175" t="inlineStr"/>
-      <c r="M175" t="inlineStr"/>
       <c r="N175" t="inlineStr">
         <is>
           <t>malla "2137" (asi se llama el punto de interrupcion en hojas 21 y 81): la lista solo da este extremo; en hoja 81 la malla sigue por las pantallas hasta 81XCM:9</t>
@@ -11950,10 +11723,6 @@
           <t>Zona hidráulica (E8)</t>
         </is>
       </c>
-      <c r="K176" t="inlineStr"/>
-      <c r="L176" t="inlineStr"/>
-      <c r="M176" t="inlineStr"/>
-      <c r="N176" t="inlineStr"/>
     </row>
     <row r="177">
       <c r="A177" t="inlineStr">
@@ -12004,10 +11773,6 @@
           <t>Zona hidráulica (E8)</t>
         </is>
       </c>
-      <c r="K177" t="inlineStr"/>
-      <c r="L177" t="inlineStr"/>
-      <c r="M177" t="inlineStr"/>
-      <c r="N177" t="inlineStr"/>
     </row>
     <row r="178">
       <c r="A178" t="inlineStr">
@@ -12058,10 +11823,6 @@
           <t>Fuera (puerta / campo)</t>
         </is>
       </c>
-      <c r="K178" t="inlineStr"/>
-      <c r="L178" t="inlineStr"/>
-      <c r="M178" t="inlineStr"/>
-      <c r="N178" t="inlineStr"/>
     </row>
     <row r="179">
       <c r="A179" t="inlineStr">
@@ -12112,10 +11873,6 @@
           <t>Fuera (puerta / campo)</t>
         </is>
       </c>
-      <c r="K179" t="inlineStr"/>
-      <c r="L179" t="inlineStr"/>
-      <c r="M179" t="inlineStr"/>
-      <c r="N179" t="inlineStr"/>
     </row>
     <row r="180">
       <c r="A180" t="inlineStr">
@@ -12166,10 +11923,6 @@
           <t>Zona hidráulica (E8)</t>
         </is>
       </c>
-      <c r="K180" t="inlineStr"/>
-      <c r="L180" t="inlineStr"/>
-      <c r="M180" t="inlineStr"/>
-      <c r="N180" t="inlineStr"/>
     </row>
     <row r="181">
       <c r="A181" t="inlineStr">
@@ -12225,7 +11978,6 @@
           <t>676.77, 530.31</t>
         </is>
       </c>
-      <c r="L181" t="inlineStr"/>
       <c r="M181" t="inlineStr">
         <is>
           <t>alta</t>
@@ -12291,7 +12043,6 @@
           <t>689.88, 499.43</t>
         </is>
       </c>
-      <c r="L182" t="inlineStr"/>
       <c r="M182" t="inlineStr">
         <is>
           <t>alta</t>
@@ -12352,9 +12103,6 @@
           <t>Zona hidráulica (E8)</t>
         </is>
       </c>
-      <c r="K183" t="inlineStr"/>
-      <c r="L183" t="inlineStr"/>
-      <c r="M183" t="inlineStr"/>
       <c r="N183" t="inlineStr">
         <is>
           <t>d2 -X1:1: EPLAN no da el pin; segun el esquema -&gt; empalme con LS001A:3 Negro</t>
@@ -12410,9 +12158,6 @@
           <t>Zona hidráulica (E8)</t>
         </is>
       </c>
-      <c r="K184" t="inlineStr"/>
-      <c r="L184" t="inlineStr"/>
-      <c r="M184" t="inlineStr"/>
       <c r="N184" t="inlineStr">
         <is>
           <t>d2 -X1:1: EPLAN no da el pin; segun el esquema -&gt; empalme con LS001A:4 Amarillo</t>
@@ -12473,7 +12218,6 @@
           <t>888.77, 641.80</t>
         </is>
       </c>
-      <c r="L185" t="inlineStr"/>
       <c r="M185" t="inlineStr">
         <is>
           <t>alta</t>
@@ -12539,7 +12283,6 @@
           <t>888.77, 629.44</t>
         </is>
       </c>
-      <c r="L186" t="inlineStr"/>
       <c r="M186" t="inlineStr">
         <is>
           <t>alta</t>
@@ -12600,7 +12343,6 @@
           <t>Bandeja principal</t>
         </is>
       </c>
-      <c r="K187" t="inlineStr"/>
       <c r="L187" t="inlineStr">
         <is>
           <t>703.95, 487.81</t>
@@ -12611,7 +12353,6 @@
           <t>alta</t>
         </is>
       </c>
-      <c r="N187" t="inlineStr"/>
     </row>
     <row r="188">
       <c r="A188" t="inlineStr">
@@ -12624,7 +12365,6 @@
           <t>Marrón</t>
         </is>
       </c>
-      <c r="C188" t="inlineStr"/>
       <c r="D188" t="inlineStr">
         <is>
           <t>E8</t>
@@ -12660,9 +12400,6 @@
           <t>Zona hidráulica (E8)</t>
         </is>
       </c>
-      <c r="K188" t="inlineStr"/>
-      <c r="L188" t="inlineStr"/>
-      <c r="M188" t="inlineStr"/>
       <c r="N188" t="inlineStr">
         <is>
           <t>d1 -X1:2: X1:2 es generico (los 4 hilos del sensor dicen X1:2); por color -&gt; empalme con el 1339 (+24V)</t>
@@ -12680,7 +12417,6 @@
           <t>Azul</t>
         </is>
       </c>
-      <c r="C189" t="inlineStr"/>
       <c r="D189" t="inlineStr">
         <is>
           <t>E8</t>
@@ -12716,9 +12452,6 @@
           <t>Zona hidráulica (E8)</t>
         </is>
       </c>
-      <c r="K189" t="inlineStr"/>
-      <c r="L189" t="inlineStr"/>
-      <c r="M189" t="inlineStr"/>
       <c r="N189" t="inlineStr">
         <is>
           <t>d1 -X1:2: X1:2 es generico (los 4 hilos del sensor dicen X1:2); por color -&gt; empalme con el 1340 (0V)</t>
@@ -12736,7 +12469,6 @@
           <t>Negro</t>
         </is>
       </c>
-      <c r="C190" t="inlineStr"/>
       <c r="D190" t="inlineStr">
         <is>
           <t>E8</t>
@@ -12772,9 +12504,6 @@
           <t>Zona hidráulica (E8)</t>
         </is>
       </c>
-      <c r="K190" t="inlineStr"/>
-      <c r="L190" t="inlineStr"/>
-      <c r="M190" t="inlineStr"/>
       <c r="N190" t="inlineStr">
         <is>
           <t>d1 -X1:2: X1:2 es generico (los 4 hilos del sensor dicen X1:2); por color -&gt; empalme con el 2166 (21PCB01:66)</t>
@@ -12792,7 +12521,6 @@
           <t>Amarillo</t>
         </is>
       </c>
-      <c r="C191" t="inlineStr"/>
       <c r="D191" t="inlineStr">
         <is>
           <t>E8</t>
@@ -12828,9 +12556,6 @@
           <t>Zona hidráulica (E8)</t>
         </is>
       </c>
-      <c r="K191" t="inlineStr"/>
-      <c r="L191" t="inlineStr"/>
-      <c r="M191" t="inlineStr"/>
       <c r="N191" t="inlineStr">
         <is>
           <t>d1 -X1:2: X1:2 es generico (los 4 hilos del sensor dicen X1:2); por color -&gt; empalme con el 2167 (21PCB01:67)</t>
@@ -12843,8 +12568,6 @@
           <t>(sin número)</t>
         </is>
       </c>
-      <c r="B192" t="inlineStr"/>
-      <c r="C192" t="inlineStr"/>
       <c r="D192" t="inlineStr">
         <is>
           <t>No es cable (puente interno)</t>
@@ -12880,9 +12603,6 @@
           <t>Bandeja principal</t>
         </is>
       </c>
-      <c r="K192" t="inlineStr"/>
-      <c r="L192" t="inlineStr"/>
-      <c r="M192" t="inlineStr"/>
       <c r="N192" t="inlineStr">
         <is>
           <t>conexion interna del rele RIF-0 (puente interno del zocalo en A2- y en 11, hoja 61); no es un cable</t>
@@ -12895,8 +12615,6 @@
           <t>(sin número)</t>
         </is>
       </c>
-      <c r="B193" t="inlineStr"/>
-      <c r="C193" t="inlineStr"/>
       <c r="D193" t="inlineStr">
         <is>
           <t>No es cable (puente interno)</t>
@@ -12932,9 +12650,6 @@
           <t>Bandeja principal</t>
         </is>
       </c>
-      <c r="K193" t="inlineStr"/>
-      <c r="L193" t="inlineStr"/>
-      <c r="M193" t="inlineStr"/>
       <c r="N193" t="inlineStr">
         <is>
           <t>conexion interna del rele RIF-0 (puente interno del zocalo en A2- y en 11, hoja 61); no es un cable</t>
@@ -12947,8 +12662,6 @@
           <t>(sin número)</t>
         </is>
       </c>
-      <c r="B194" t="inlineStr"/>
-      <c r="C194" t="inlineStr"/>
       <c r="D194" t="inlineStr">
         <is>
           <t>No es cable (puente interno)</t>
@@ -12984,9 +12697,6 @@
           <t>Bandeja principal</t>
         </is>
       </c>
-      <c r="K194" t="inlineStr"/>
-      <c r="L194" t="inlineStr"/>
-      <c r="M194" t="inlineStr"/>
       <c r="N194" t="inlineStr">
         <is>
           <t>conexion interna del rele RIF-0 (puente interno del zocalo en A2- y en 11, hoja 61); no es un cable</t>
@@ -12999,8 +12709,6 @@
           <t>(sin número)</t>
         </is>
       </c>
-      <c r="B195" t="inlineStr"/>
-      <c r="C195" t="inlineStr"/>
       <c r="D195" t="inlineStr">
         <is>
           <t>No es cable (puente interno)</t>
@@ -13036,9 +12744,6 @@
           <t>Bandeja principal</t>
         </is>
       </c>
-      <c r="K195" t="inlineStr"/>
-      <c r="L195" t="inlineStr"/>
-      <c r="M195" t="inlineStr"/>
       <c r="N195" t="inlineStr">
         <is>
           <t>conexion interna del rele RIF-0 (puente interno del zocalo en A2- y en 11, hoja 61); no es un cable</t>
@@ -13175,12 +12880,12 @@
       </c>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>Se mapeó L / PE / N de izquierda a derecha (según el símbolo). La hoja 8 no rotula los tornillos; con la norma china podría ser N / PE / L.</t>
+          <t>Corregido el 2026-10-07 por el taller: N / PE / L de izquierda a derecha, como la foto oficial de Phoenix. El 1182 (N) va al tornillo de la izquierda y el 1181 (L) al de la derecha.</t>
         </is>
       </c>
       <c r="C7" s="5" t="inlineStr">
         <is>
-          <t>Confirmar con el toma real.</t>
+          <t>Nada (resuelto).</t>
         </is>
       </c>
     </row>

</xml_diff>